<commit_message>
feat(web): implementar cockpit executivo 5D com 8 visoes integradas, apis e documentacao mestre
</commit_message>
<xml_diff>
--- a/projetos/OBRA_TMULT/04_PRODUCAO_E_AVANCO/PAINEL_RDOS_OBRA.xlsx
+++ b/projetos/OBRA_TMULT/04_PRODUCAO_E_AVANCO/PAINEL_RDOS_OBRA.xlsx
@@ -156,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -236,6 +236,25 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -919,7 +938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1431,6 +1450,70 @@
         </is>
       </c>
     </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="37" t="inlineStr">
+        <is>
+          <t>RDO-008</t>
+        </is>
+      </c>
+      <c r="B11" s="37" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="C11" s="38" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>Ensolarado</t>
+        </is>
+      </c>
+      <c r="E11" s="38" t="inlineStr">
+        <is>
+          <t>Ensolarado</t>
+        </is>
+      </c>
+      <c r="F11" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="40" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" s="40" t="n">
+        <v>16</v>
+      </c>
+      <c r="I11" s="41">
+        <f>G11+H11</f>
+        <v/>
+      </c>
+      <c r="J11" s="42">
+        <f>(I11*8.8)-(F11*I11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="38" t="inlineStr">
+        <is>
+          <t>EAP 1.3 / Fundações e Estrutura</t>
+        </is>
+      </c>
+      <c r="L11" s="38" t="inlineStr">
+        <is>
+          <t>FVS-02</t>
+        </is>
+      </c>
+      <c r="M11" s="43" t="inlineStr">
+        <is>
+          <t>🟢 Aprovado</t>
+        </is>
+      </c>
+      <c r="N11" s="38" t="inlineStr">
+        <is>
+          <t>RDO 11/09/2026: 8 pedreiros, 6 serventes e 2 carpinteiros. Clima de sol manha e tarde. Escavacao sapatas S21 a S28. FVS-02 aprovada com sucesso. Sem paralisacoes.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>

</xml_diff>